<commit_message>
fix: update BVA order payment
</commit_message>
<xml_diff>
--- a/docs/testing/BVA/order & payment/Testcase_BVA_Order_Payment.xlsx
+++ b/docs/testing/BVA/order & payment/Testcase_BVA_Order_Payment.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="144">
   <si>
     <t>Biến đầu vào</t>
   </si>
@@ -526,7 +526,10 @@
 total = 4.999.950.000đ, discount = 500đ, final = 4.999.949.500đ.</t>
   </si>
   <si>
-    <t>HTTP 201 Created. Đạt yêu cầu đơn giá lân cận tối đa.</t>
+    <t>HTTP 400 Bad Request. Hệ thống báo lỗi "numeric field overflow" do cột tiền tệ DECIMAL(10,2) trong Database bị tràn số khi tổng tiền đạt mức 4.999.950.000đ (~5 Tỷ VNĐ).</t>
+  </si>
+  <si>
+    <t>FAIL</t>
   </si>
   <si>
     <t>TC_BVA_S_04</t>
@@ -549,7 +552,7 @@
 total = 5.000.000.000đ, discount = 500đ, final = 4.999.999.500đ.</t>
   </si>
   <si>
-    <t>HTTP 201 Created. Đạt yêu cầu đơn giá biên tối đa 100M.</t>
+    <t>HTTP 400 Bad Request. Hệ thống báo lỗi "numeric field overflow" do cột tiền tệ DECIMAL(10,2) trong Database bị tràn số khi tổng tiền đạt mức 5.000.000.000đ (5 Tỷ VNĐ).</t>
   </si>
 </sst>
 </file>
@@ -562,7 +565,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="30">
+  <fonts count="31">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -609,6 +612,13 @@
       <charset val="134"/>
     </font>
     <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Segoe UI"/>
+      <charset val="134"/>
+    </font>
+    <font>
       <sz val="9"/>
       <name val="Arial"/>
       <charset val="134"/>
@@ -778,7 +788,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="38">
+  <fills count="39">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -800,6 +810,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD4EFDF"/>
+        <bgColor rgb="FFD4EFDF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.4"/>
         <bgColor rgb="FFD4EFDF"/>
       </patternFill>
     </fill>
@@ -1141,55 +1157,52 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1204,74 +1217,77 @@
     <xf numFmtId="0" fontId="29" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1300,16 +1316,19 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1318,7 +1337,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1706,71 +1725,71 @@
       </c>
     </row>
     <row r="2" s="1" customFormat="1" ht="25" customHeight="1" spans="1:7">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="17">
+      <c r="B2" s="18">
         <v>1</v>
       </c>
-      <c r="C2" s="17">
+      <c r="C2" s="18">
         <v>2</v>
       </c>
-      <c r="D2" s="17">
+      <c r="D2" s="18">
         <v>50</v>
       </c>
-      <c r="E2" s="17">
+      <c r="E2" s="18">
         <v>98</v>
       </c>
-      <c r="F2" s="17">
+      <c r="F2" s="18">
         <v>99</v>
       </c>
-      <c r="G2" s="18" t="s">
+      <c r="G2" s="19" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="3" s="1" customFormat="1" ht="25" customHeight="1" spans="1:7">
-      <c r="A3" s="16" t="s">
+      <c r="A3" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="17">
+      <c r="B3" s="18">
         <v>0</v>
       </c>
-      <c r="C3" s="17">
+      <c r="C3" s="18">
         <v>1</v>
       </c>
-      <c r="D3" s="17">
+      <c r="D3" s="18">
         <v>500</v>
       </c>
-      <c r="E3" s="17">
+      <c r="E3" s="18">
         <v>7499999</v>
       </c>
-      <c r="F3" s="17">
+      <c r="F3" s="18">
         <v>7500000</v>
       </c>
-      <c r="G3" s="18" t="s">
+      <c r="G3" s="19" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="4" s="1" customFormat="1" ht="25" customHeight="1" spans="1:7">
-      <c r="A4" s="16" t="s">
+      <c r="A4" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="17" t="s">
+      <c r="B4" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="17" t="s">
+      <c r="C4" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="17" t="s">
+      <c r="D4" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="17" t="s">
+      <c r="E4" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="F4" s="17" t="s">
+      <c r="F4" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="G4" s="18" t="s">
+      <c r="G4" s="19" t="s">
         <v>17</v>
       </c>
     </row>
@@ -2328,22 +2347,22 @@
       <c r="K14" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="L14" s="11" t="s">
-        <v>41</v>
+      <c r="L14" s="12" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="15" s="1" customFormat="1" ht="55" customHeight="1" spans="1:12">
       <c r="A15" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>43</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E15" s="6" t="s">
         <v>34</v>
@@ -2352,239 +2371,239 @@
         <v>46</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="I15" s="10" t="s">
         <v>49</v>
       </c>
       <c r="J15" s="7" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="K15" s="7" t="s">
-        <v>142</v>
-      </c>
-      <c r="L15" s="11" t="s">
-        <v>41</v>
+        <v>143</v>
+      </c>
+      <c r="L15" s="12" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="16" ht="42" customHeight="1" spans="1:12">
-      <c r="A16" s="12"/>
-      <c r="B16" s="12"/>
-      <c r="C16" s="13"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="12"/>
-      <c r="F16" s="13"/>
-      <c r="G16" s="13"/>
-      <c r="H16" s="13"/>
-      <c r="K16" s="13"/>
-      <c r="L16" s="15"/>
+      <c r="A16" s="13"/>
+      <c r="B16" s="13"/>
+      <c r="C16" s="14"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="13"/>
+      <c r="F16" s="14"/>
+      <c r="G16" s="14"/>
+      <c r="H16" s="14"/>
+      <c r="K16" s="14"/>
+      <c r="L16" s="16"/>
     </row>
     <row r="17" ht="42" customHeight="1" spans="1:12">
-      <c r="A17" s="12"/>
-      <c r="B17" s="12"/>
-      <c r="C17" s="13"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="12"/>
-      <c r="F17" s="13"/>
-      <c r="G17" s="13"/>
-      <c r="H17" s="13"/>
-      <c r="K17" s="13"/>
-      <c r="L17" s="15"/>
+      <c r="A17" s="13"/>
+      <c r="B17" s="13"/>
+      <c r="C17" s="14"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="13"/>
+      <c r="F17" s="14"/>
+      <c r="G17" s="14"/>
+      <c r="H17" s="14"/>
+      <c r="K17" s="14"/>
+      <c r="L17" s="16"/>
     </row>
     <row r="18" ht="42" customHeight="1" spans="1:12">
-      <c r="A18" s="12"/>
-      <c r="B18" s="12"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="12"/>
-      <c r="F18" s="13"/>
-      <c r="G18" s="13"/>
-      <c r="H18" s="13"/>
-      <c r="K18" s="13"/>
-      <c r="L18" s="15"/>
+      <c r="A18" s="13"/>
+      <c r="B18" s="13"/>
+      <c r="C18" s="14"/>
+      <c r="D18" s="15"/>
+      <c r="E18" s="13"/>
+      <c r="F18" s="14"/>
+      <c r="G18" s="14"/>
+      <c r="H18" s="14"/>
+      <c r="K18" s="14"/>
+      <c r="L18" s="16"/>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:12">
-      <c r="A19" s="12"/>
-      <c r="B19" s="12"/>
-      <c r="C19" s="13"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="13"/>
-      <c r="G19" s="13"/>
-      <c r="H19" s="13"/>
-      <c r="K19" s="13"/>
-      <c r="L19" s="15"/>
+      <c r="A19" s="13"/>
+      <c r="B19" s="13"/>
+      <c r="C19" s="14"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="13"/>
+      <c r="F19" s="14"/>
+      <c r="G19" s="14"/>
+      <c r="H19" s="14"/>
+      <c r="K19" s="14"/>
+      <c r="L19" s="16"/>
     </row>
     <row r="20" ht="42" customHeight="1" spans="1:12">
-      <c r="A20" s="12"/>
-      <c r="B20" s="12"/>
-      <c r="C20" s="13"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="12"/>
-      <c r="F20" s="13"/>
-      <c r="G20" s="13"/>
-      <c r="H20" s="13"/>
-      <c r="K20" s="13"/>
-      <c r="L20" s="15"/>
+      <c r="A20" s="13"/>
+      <c r="B20" s="13"/>
+      <c r="C20" s="14"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="13"/>
+      <c r="F20" s="14"/>
+      <c r="G20" s="14"/>
+      <c r="H20" s="14"/>
+      <c r="K20" s="14"/>
+      <c r="L20" s="16"/>
     </row>
     <row r="21" ht="42" customHeight="1" spans="1:12">
-      <c r="A21" s="12"/>
-      <c r="B21" s="12"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="12"/>
-      <c r="F21" s="13"/>
-      <c r="G21" s="13"/>
-      <c r="H21" s="13"/>
-      <c r="K21" s="13"/>
-      <c r="L21" s="15"/>
+      <c r="A21" s="13"/>
+      <c r="B21" s="13"/>
+      <c r="C21" s="14"/>
+      <c r="D21" s="15"/>
+      <c r="E21" s="13"/>
+      <c r="F21" s="14"/>
+      <c r="G21" s="14"/>
+      <c r="H21" s="14"/>
+      <c r="K21" s="14"/>
+      <c r="L21" s="16"/>
     </row>
     <row r="22" ht="42" customHeight="1" spans="1:12">
-      <c r="A22" s="12"/>
-      <c r="B22" s="12"/>
-      <c r="C22" s="13"/>
-      <c r="D22" s="14"/>
-      <c r="E22" s="12"/>
-      <c r="F22" s="13"/>
-      <c r="G22" s="13"/>
-      <c r="H22" s="13"/>
-      <c r="K22" s="13"/>
-      <c r="L22" s="15"/>
+      <c r="A22" s="13"/>
+      <c r="B22" s="13"/>
+      <c r="C22" s="14"/>
+      <c r="D22" s="15"/>
+      <c r="E22" s="13"/>
+      <c r="F22" s="14"/>
+      <c r="G22" s="14"/>
+      <c r="H22" s="14"/>
+      <c r="K22" s="14"/>
+      <c r="L22" s="16"/>
     </row>
     <row r="23" ht="42" customHeight="1" spans="1:12">
-      <c r="A23" s="12"/>
-      <c r="B23" s="12"/>
-      <c r="C23" s="13"/>
-      <c r="D23" s="14"/>
-      <c r="E23" s="12"/>
-      <c r="F23" s="13"/>
-      <c r="G23" s="13"/>
-      <c r="H23" s="13"/>
-      <c r="K23" s="13"/>
-      <c r="L23" s="15"/>
+      <c r="A23" s="13"/>
+      <c r="B23" s="13"/>
+      <c r="C23" s="14"/>
+      <c r="D23" s="15"/>
+      <c r="E23" s="13"/>
+      <c r="F23" s="14"/>
+      <c r="G23" s="14"/>
+      <c r="H23" s="14"/>
+      <c r="K23" s="14"/>
+      <c r="L23" s="16"/>
     </row>
     <row r="24" ht="42" customHeight="1" spans="1:12">
-      <c r="A24" s="12"/>
-      <c r="B24" s="12"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="14"/>
-      <c r="E24" s="12"/>
-      <c r="F24" s="13"/>
-      <c r="G24" s="13"/>
-      <c r="H24" s="13"/>
-      <c r="K24" s="13"/>
-      <c r="L24" s="15"/>
+      <c r="A24" s="13"/>
+      <c r="B24" s="13"/>
+      <c r="C24" s="14"/>
+      <c r="D24" s="15"/>
+      <c r="E24" s="13"/>
+      <c r="F24" s="14"/>
+      <c r="G24" s="14"/>
+      <c r="H24" s="14"/>
+      <c r="K24" s="14"/>
+      <c r="L24" s="16"/>
     </row>
     <row r="25" ht="42" customHeight="1" spans="1:12">
-      <c r="A25" s="12"/>
-      <c r="B25" s="12"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="14"/>
-      <c r="E25" s="12"/>
-      <c r="F25" s="13"/>
-      <c r="G25" s="13"/>
-      <c r="H25" s="13"/>
-      <c r="K25" s="13"/>
-      <c r="L25" s="15"/>
+      <c r="A25" s="13"/>
+      <c r="B25" s="13"/>
+      <c r="C25" s="14"/>
+      <c r="D25" s="15"/>
+      <c r="E25" s="13"/>
+      <c r="F25" s="14"/>
+      <c r="G25" s="14"/>
+      <c r="H25" s="14"/>
+      <c r="K25" s="14"/>
+      <c r="L25" s="16"/>
     </row>
     <row r="26" ht="42" customHeight="1" spans="1:12">
-      <c r="A26" s="12"/>
-      <c r="B26" s="12"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="14"/>
-      <c r="E26" s="12"/>
-      <c r="F26" s="13"/>
-      <c r="G26" s="13"/>
-      <c r="H26" s="13"/>
-      <c r="K26" s="13"/>
-      <c r="L26" s="15"/>
+      <c r="A26" s="13"/>
+      <c r="B26" s="13"/>
+      <c r="C26" s="14"/>
+      <c r="D26" s="15"/>
+      <c r="E26" s="13"/>
+      <c r="F26" s="14"/>
+      <c r="G26" s="14"/>
+      <c r="H26" s="14"/>
+      <c r="K26" s="14"/>
+      <c r="L26" s="16"/>
     </row>
     <row r="27" ht="42" customHeight="1" spans="1:12">
-      <c r="A27" s="12"/>
-      <c r="B27" s="12"/>
-      <c r="C27" s="13"/>
-      <c r="D27" s="14"/>
-      <c r="E27" s="12"/>
-      <c r="F27" s="13"/>
-      <c r="G27" s="13"/>
-      <c r="H27" s="13"/>
-      <c r="K27" s="13"/>
-      <c r="L27" s="15"/>
+      <c r="A27" s="13"/>
+      <c r="B27" s="13"/>
+      <c r="C27" s="14"/>
+      <c r="D27" s="15"/>
+      <c r="E27" s="13"/>
+      <c r="F27" s="14"/>
+      <c r="G27" s="14"/>
+      <c r="H27" s="14"/>
+      <c r="K27" s="14"/>
+      <c r="L27" s="16"/>
     </row>
     <row r="28" ht="42" customHeight="1" spans="1:12">
-      <c r="A28" s="12"/>
-      <c r="B28" s="12"/>
-      <c r="C28" s="13"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="12"/>
-      <c r="F28" s="13"/>
-      <c r="G28" s="13"/>
-      <c r="H28" s="13"/>
-      <c r="K28" s="13"/>
-      <c r="L28" s="15"/>
+      <c r="A28" s="13"/>
+      <c r="B28" s="13"/>
+      <c r="C28" s="14"/>
+      <c r="D28" s="15"/>
+      <c r="E28" s="13"/>
+      <c r="F28" s="14"/>
+      <c r="G28" s="14"/>
+      <c r="H28" s="14"/>
+      <c r="K28" s="14"/>
+      <c r="L28" s="16"/>
     </row>
     <row r="29" ht="42" customHeight="1" spans="1:12">
-      <c r="A29" s="12"/>
-      <c r="B29" s="12"/>
-      <c r="C29" s="13"/>
-      <c r="D29" s="14"/>
-      <c r="E29" s="12"/>
-      <c r="F29" s="13"/>
-      <c r="G29" s="13"/>
-      <c r="H29" s="13"/>
-      <c r="K29" s="13"/>
-      <c r="L29" s="15"/>
+      <c r="A29" s="13"/>
+      <c r="B29" s="13"/>
+      <c r="C29" s="14"/>
+      <c r="D29" s="15"/>
+      <c r="E29" s="13"/>
+      <c r="F29" s="14"/>
+      <c r="G29" s="14"/>
+      <c r="H29" s="14"/>
+      <c r="K29" s="14"/>
+      <c r="L29" s="16"/>
     </row>
     <row r="30" ht="42" customHeight="1" spans="1:12">
-      <c r="A30" s="12"/>
-      <c r="B30" s="12"/>
-      <c r="C30" s="13"/>
-      <c r="D30" s="14"/>
-      <c r="E30" s="12"/>
-      <c r="F30" s="13"/>
-      <c r="G30" s="13"/>
-      <c r="H30" s="13"/>
-      <c r="K30" s="13"/>
-      <c r="L30" s="15"/>
+      <c r="A30" s="13"/>
+      <c r="B30" s="13"/>
+      <c r="C30" s="14"/>
+      <c r="D30" s="15"/>
+      <c r="E30" s="13"/>
+      <c r="F30" s="14"/>
+      <c r="G30" s="14"/>
+      <c r="H30" s="14"/>
+      <c r="K30" s="14"/>
+      <c r="L30" s="16"/>
     </row>
     <row r="31" ht="42" customHeight="1" spans="1:12">
-      <c r="A31" s="12"/>
-      <c r="B31" s="12"/>
-      <c r="C31" s="13"/>
-      <c r="D31" s="14"/>
-      <c r="E31" s="12"/>
-      <c r="F31" s="13"/>
-      <c r="G31" s="13"/>
-      <c r="H31" s="13"/>
-      <c r="K31" s="13"/>
-      <c r="L31" s="15"/>
+      <c r="A31" s="13"/>
+      <c r="B31" s="13"/>
+      <c r="C31" s="14"/>
+      <c r="D31" s="15"/>
+      <c r="E31" s="13"/>
+      <c r="F31" s="14"/>
+      <c r="G31" s="14"/>
+      <c r="H31" s="14"/>
+      <c r="K31" s="14"/>
+      <c r="L31" s="16"/>
     </row>
     <row r="32" ht="42" customHeight="1" spans="1:12">
-      <c r="A32" s="12"/>
-      <c r="B32" s="12"/>
-      <c r="C32" s="13"/>
-      <c r="D32" s="14"/>
-      <c r="E32" s="12"/>
-      <c r="F32" s="13"/>
-      <c r="G32" s="13"/>
-      <c r="H32" s="13"/>
-      <c r="K32" s="13"/>
-      <c r="L32" s="15"/>
+      <c r="A32" s="13"/>
+      <c r="B32" s="13"/>
+      <c r="C32" s="14"/>
+      <c r="D32" s="15"/>
+      <c r="E32" s="13"/>
+      <c r="F32" s="14"/>
+      <c r="G32" s="14"/>
+      <c r="H32" s="14"/>
+      <c r="K32" s="14"/>
+      <c r="L32" s="16"/>
     </row>
     <row r="33" ht="42" customHeight="1" spans="1:12">
-      <c r="A33" s="12"/>
-      <c r="B33" s="12"/>
-      <c r="C33" s="13"/>
-      <c r="D33" s="14"/>
-      <c r="E33" s="12"/>
-      <c r="F33" s="13"/>
-      <c r="G33" s="13"/>
-      <c r="H33" s="13"/>
-      <c r="K33" s="13"/>
-      <c r="L33" s="15"/>
+      <c r="A33" s="13"/>
+      <c r="B33" s="13"/>
+      <c r="C33" s="14"/>
+      <c r="D33" s="15"/>
+      <c r="E33" s="13"/>
+      <c r="F33" s="14"/>
+      <c r="G33" s="14"/>
+      <c r="H33" s="14"/>
+      <c r="K33" s="14"/>
+      <c r="L33" s="16"/>
     </row>
   </sheetData>
   <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:L33" etc:filterBottomFollowUsedRange="0">

</xml_diff>